<commit_message>
research: add original feedback text fields
</commit_message>
<xml_diff>
--- a/outputs/01a064d5-0ee8-7482-8ace-77518f64e0fa/uae-competitor-feedback-pilot.xlsx
+++ b/outputs/01a064d5-0ee8-7482-8ace-77518f64e0fa/uae-competitor-feedback-pilot.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Summary" sheetId="1" r:id="Rcf4b3e6dd307485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Country &amp; Language" sheetId="2" r:id="Rc8338b0e8e504cd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Feasibility" sheetId="3" r:id="Re86f67ff35ff4d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query Log" sheetId="4" r:id="Rc0df521453344b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Feedback" sheetId="5" r:id="R528df231763543f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coded Feedback" sheetId="6" r:id="R7cd3f73dc4454fd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Matrix" sheetId="7" r:id="R3a07e4466c124285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="8" r:id="R899bb27caa3f4c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot Summary" sheetId="1" r:id="R62716c707f5f4442"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Country &amp; Language" sheetId="2" r:id="R15ddfcaac80f494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Feasibility" sheetId="3" r:id="Re45a2784fb674458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query Log" sheetId="4" r:id="Rd4586ea6ce044dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Feedback" sheetId="5" r:id="R58a6055ae6084c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coded Feedback" sheetId="6" r:id="R0b64362f1a22474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Matrix" sheetId="7" r:id="R2c0db67766ac4a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="8" r:id="R03214b43158344cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={26D3EE28-5DBA-4BD0-9308-FB4BA5601ECD}</x:author>
+    <x:author>tc={F3EAEB3C-D55B-486B-80FE-9904341E4D6E}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="E5" authorId="0">
@@ -37,7 +37,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={E31C0237-F99C-495F-BC91-0C551DD4EE04}</x:author>
+    <x:author>tc={874A7CA6-8AAF-484C-A700-667AD2DC489D}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="D5" authorId="0">
@@ -658,7 +658,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{356925B2-BC65-44AF-8C14-8A7662C10055}"/>
+  <xltc:person displayName="User" id="{A2193874-D188-454C-BC13-0F71F53D33A5}"/>
 </xltc:personList>
 </file>
 
@@ -727,8 +727,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RawFeedbackTable" displayName="RawFeedbackTable" ref="A4:AF24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="32">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RawFeedbackTable" displayName="RawFeedbackTable" ref="A4:AH24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="34">
     <x:tableColumn id="1" name="feedback_id"/>
     <x:tableColumn id="2" name="product"/>
     <x:tableColumn id="3" name="product_scope"/>
@@ -756,11 +756,13 @@
     <x:tableColumn id="25" name="switching_signal"/>
     <x:tableColumn id="26" name="sentiment"/>
     <x:tableColumn id="27" name="capture_mode"/>
-    <x:tableColumn id="28" name="evidence_excerpt"/>
-    <x:tableColumn id="29" name="inclusion_status"/>
-    <x:tableColumn id="30" name="exclusion_reason"/>
-    <x:tableColumn id="31" name="duplicate_group"/>
-    <x:tableColumn id="32" name="researcher_note"/>
+    <x:tableColumn id="28" name="original_text"/>
+    <x:tableColumn id="29" name="original_text_translation_cn"/>
+    <x:tableColumn id="30" name="evidence_excerpt"/>
+    <x:tableColumn id="31" name="inclusion_status"/>
+    <x:tableColumn id="32" name="exclusion_reason"/>
+    <x:tableColumn id="33" name="duplicate_group"/>
+    <x:tableColumn id="34" name="researcher_note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1049,7 +1051,7 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="E5" dT="2026-09-03T21:24:10.55" personId="{356925B2-BC65-44AF-8C14-8A7662C10055}" id="{26D3EE28-5DBA-4BD0-9308-FB4BA5601ECD}">
+  <xltc:threadedComment ref="E5" dT="2026-09-03T23:53:44.143" personId="{A2193874-D188-454C-BC13-0F71F53D33A5}" id="{F3EAEB3C-D55B-486B-80FE-9904341E4D6E}">
     <xltc:text>High geo means explicit source profile/body location evidence; it is not independent identity verification.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1057,7 +1059,7 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="D5" dT="2026-09-03T21:24:10.55" personId="{356925B2-BC65-44AF-8C14-8A7662C10055}" id="{E31C0237-F99C-495F-BC91-0C551DD4EE04}">
+  <xltc:threadedComment ref="D5" dT="2026-09-03T23:53:44.145" personId="{A2193874-D188-454C-BC13-0F71F53D33A5}" id="{874A7CA6-8AAF-484C-A700-667AD2DC489D}">
     <xltc:text>Arabic is a query language, never a substitute for country attribution.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1394,7 +1396,7 @@
     <x:mergeCell ref="A21:H23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829486079ff94fff"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8de6cf098244e8d"/>
 </x:worksheet>
 </file>
 
@@ -1740,9 +1742,9 @@
     <x:mergeCell ref="A10:L10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c409dd6f55345d3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95cdf1730be84e76"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raac7b3f3dfcf48a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fffbbdc0ace485b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2444,7 +2446,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8df302ec744bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82d4ab5c7c21453f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3390,7 +3392,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f0ebdb7ab514259"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689758fa12c94cc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3427,10 +3429,12 @@
     <x:col min="26" max="26" width="12" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="30" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="42" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="23" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="32" hidden="0" customWidth="1"/>
-    <x:col min="31" max="31" width="16" hidden="0" customWidth="1"/>
-    <x:col min="32" max="32" width="38" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="42" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="42" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="23" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="32" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="16" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -3530,10 +3534,16 @@
       <x:c r="AF1" s="3" t="str">
         <x:v>Raw Feedback｜20 条发现记录（含排除与分流）</x:v>
       </x:c>
+      <x:c r="AG1" s="3" t="str">
+        <x:v>Raw Feedback｜20 条发现记录（含排除与分流）</x:v>
+      </x:c>
+      <x:c r="AH1" s="3" t="str">
+        <x:v>Raw Feedback｜20 条发现记录（含排除与分流）</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="24" t="str">
-        <x:v>保留原始发现层，不把语言或 UAE storefront 自动转换成 UAE 用户；evidence_excerpt 均为研究员短转述，原链接用于复核。</x:v>
+        <x:v>original_text 保存可核验的最短原文证据片段，original_text_translation_cn 为中文翻译；空白表示未可靠取得，不用研究员转述冒充原话。</x:v>
       </x:c>
       <x:c r="B2" s="24"/>
       <x:c r="C2" s="24"/>
@@ -3566,6 +3576,8 @@
       <x:c r="AD2" s="24"/>
       <x:c r="AE2" s="24"/>
       <x:c r="AF2" s="24"/>
+      <x:c r="AG2" s="24"/>
+      <x:c r="AH2" s="24"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="15" t="str">
@@ -3650,22 +3662,28 @@
         <x:v>capture_mode</x:v>
       </x:c>
       <x:c r="AB4" s="16" t="str">
+        <x:v>original_text</x:v>
+      </x:c>
+      <x:c r="AC4" s="16" t="str">
+        <x:v>original_text_translation_cn</x:v>
+      </x:c>
+      <x:c r="AD4" s="16" t="str">
         <x:v>evidence_excerpt</x:v>
       </x:c>
-      <x:c r="AC4" s="16" t="str">
+      <x:c r="AE4" s="16" t="str">
         <x:v>inclusion_status</x:v>
       </x:c>
-      <x:c r="AD4" s="16" t="str">
+      <x:c r="AF4" s="16" t="str">
         <x:v>exclusion_reason</x:v>
       </x:c>
-      <x:c r="AE4" s="16" t="str">
+      <x:c r="AG4" s="16" t="str">
         <x:v>duplicate_group</x:v>
       </x:c>
-      <x:c r="AF4" s="17" t="str">
+      <x:c r="AH4" s="17" t="str">
         <x:v>researcher_note</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="74" customHeight="1">
+    <x:row r="5" ht="82" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>FB-ARE-20260602-000001</x:v>
       </x:c>
@@ -3748,18 +3766,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB5" s="19" t="str">
+        <x:v>Llevo gastando más de 200 dólares en créditos</x:v>
+      </x:c>
+      <x:c r="AC5" s="19" t="str">
+        <x:v>我已经在积分上花了超过 200 美元。</x:v>
+      </x:c>
+      <x:c r="AD5" s="19" t="str">
         <x:v>[转述] 应用已做得较深，但积分与退款问题造成锁定</x:v>
       </x:c>
-      <x:c r="AC5" s="19" t="str">
+      <x:c r="AE5" s="19" t="str">
         <x:v>Included-Core</x:v>
       </x:c>
-      <x:c r="AD5" s="19" t="str"/>
-      <x:c r="AE5" s="19" t="str"/>
-      <x:c r="AF5" s="19" t="str">
+      <x:c r="AF5" s="19" t="str"/>
+      <x:c r="AG5" s="19" t="str"/>
+      <x:c r="AH5" s="19" t="str">
         <x:v>国家来自平台资料标识，未独立验证身份</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="74" customHeight="1">
+    <x:row r="6" ht="82" customHeight="1">
       <x:c r="A6" s="19" t="str">
         <x:v>FB-ARE-20260815-000002</x:v>
       </x:c>
@@ -3840,18 +3864,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB6" s="19" t="str">
+        <x:v>prepare presentations for top management on a very short time frame</x:v>
+      </x:c>
+      <x:c r="AC6" s="19" t="str">
+        <x:v>在很短时间内为高层准备演示材料。</x:v>
+      </x:c>
+      <x:c r="AD6" s="19" t="str">
         <x:v>[转述] Super Agent 帮助在短时限内完成高层演示</x:v>
       </x:c>
-      <x:c r="AC6" s="19" t="str">
+      <x:c r="AE6" s="19" t="str">
         <x:v>Included-Core</x:v>
       </x:c>
-      <x:c r="AD6" s="19" t="str"/>
-      <x:c r="AE6" s="19" t="str"/>
-      <x:c r="AF6" s="19" t="str">
+      <x:c r="AF6" s="19" t="str"/>
+      <x:c r="AG6" s="19" t="str"/>
+      <x:c r="AH6" s="19" t="str">
         <x:v>任务和结果明确；角色仍为推断性标签</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="74" customHeight="1">
+    <x:row r="7" ht="82" customHeight="1">
       <x:c r="A7" s="19" t="str">
         <x:v>FB-ARE-20260707-000003</x:v>
       </x:c>
@@ -3934,18 +3964,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB7" s="19" t="str">
+        <x:v>building presentations, creating spreadsheets, managing CRM dashboards</x:v>
+      </x:c>
+      <x:c r="AC7" s="19" t="str">
+        <x:v>制作演示、创建表格并管理 CRM 仪表盘。</x:v>
+      </x:c>
+      <x:c r="AD7" s="19" t="str">
         <x:v>[转述] 创始人用它统一演示、表格、CRM 与内容工作</x:v>
       </x:c>
-      <x:c r="AC7" s="19" t="str">
+      <x:c r="AE7" s="19" t="str">
         <x:v>Included-Core</x:v>
       </x:c>
-      <x:c r="AD7" s="19" t="str"/>
-      <x:c r="AE7" s="19" t="str"/>
-      <x:c r="AF7" s="19" t="str">
+      <x:c r="AF7" s="19" t="str"/>
+      <x:c r="AG7" s="19" t="str"/>
+      <x:c r="AH7" s="19" t="str">
         <x:v>高信息密度正向留存样本</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="74" customHeight="1">
+    <x:row r="8" ht="82" customHeight="1">
       <x:c r="A8" s="19" t="str">
         <x:v>FB-ARE-20260419-000004</x:v>
       </x:c>
@@ -4028,18 +4064,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB8" s="19" t="str">
+        <x:v>generate a simple ZIP file containing my designs</x:v>
+      </x:c>
+      <x:c r="AC8" s="19" t="str">
+        <x:v>生成一个包含我的设计文件的简单 ZIP。</x:v>
+      </x:c>
+      <x:c r="AD8" s="19" t="str">
         <x:v>[转述] ZIP 与透明 logo 任务失败，过程中持续扣积分</x:v>
       </x:c>
-      <x:c r="AC8" s="19" t="str">
+      <x:c r="AE8" s="19" t="str">
         <x:v>Included-Core</x:v>
       </x:c>
-      <x:c r="AD8" s="19" t="str"/>
-      <x:c r="AE8" s="19" t="str"/>
-      <x:c r="AF8" s="19" t="str">
+      <x:c r="AF8" s="19" t="str"/>
+      <x:c r="AG8" s="19" t="str"/>
+      <x:c r="AH8" s="19" t="str">
         <x:v>可明确编码失败阶段、结果和成本</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="74" customHeight="1">
+    <x:row r="9" ht="82" customHeight="1">
       <x:c r="A9" s="19" t="str">
         <x:v>FB-ARE-20260804-000005</x:v>
       </x:c>
@@ -4122,18 +4164,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB9" s="19" t="str">
+        <x:v>investigate and refund appropriately</x:v>
+      </x:c>
+      <x:c r="AC9" s="19" t="str">
+        <x:v>进行调查并适当退款。</x:v>
+      </x:c>
+      <x:c r="AD9" s="19" t="str">
         <x:v>[转述] credits 争议得到调查与退款</x:v>
       </x:c>
-      <x:c r="AC9" s="19" t="str">
+      <x:c r="AE9" s="19" t="str">
         <x:v>Included-Adjacent</x:v>
       </x:c>
-      <x:c r="AD9" s="19" t="str"/>
-      <x:c r="AE9" s="19" t="str"/>
-      <x:c r="AF9" s="19" t="str">
+      <x:c r="AF9" s="19" t="str"/>
+      <x:c r="AG9" s="19" t="str"/>
+      <x:c r="AH9" s="19" t="str">
         <x:v>能评价售后但缺少具体 Cowork 工作任务</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="74" customHeight="1">
+    <x:row r="10" ht="82" customHeight="1">
       <x:c r="A10" s="19" t="str">
         <x:v>FB-ARE-20260722-000006</x:v>
       </x:c>
@@ -4216,18 +4264,24 @@
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
       <x:c r="AB10" s="19" t="str">
+        <x:v>I canceled my subscription in May 2026 and they still charged me</x:v>
+      </x:c>
+      <x:c r="AC10" s="19" t="str">
+        <x:v>我在 2026 年 5 月取消订阅，但他们仍继续扣费。</x:v>
+      </x:c>
+      <x:c r="AD10" s="19" t="str">
         <x:v>[转述] 取消后仍连续扣费，且无法获得人工支持</x:v>
       </x:c>
-      <x:c r="AC10" s="19" t="str">
+      <x:c r="AE10" s="19" t="str">
         <x:v>Included-Adjacent</x:v>
       </x:c>
-      <x:c r="AD10" s="19" t="str"/>
-      <x:c r="AE10" s="19" t="str"/>
-      <x:c r="AF10" s="19" t="str">
+      <x:c r="AF10" s="19" t="str"/>
+      <x:c r="AG10" s="19" t="str"/>
+      <x:c r="AH10" s="19" t="str">
         <x:v>不是 Comet/Cowork 任务反馈，只进入商业系统边界</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="74" customHeight="1">
+    <x:row r="11" ht="82" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>FB-ARE-20260809-000007</x:v>
       </x:c>
@@ -4307,21 +4361,23 @@
       <x:c r="AA11" s="19" t="str">
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
-      <x:c r="AB11" s="19" t="str">
+      <x:c r="AB11" s="19" t="str"/>
+      <x:c r="AC11" s="19" t="str"/>
+      <x:c r="AD11" s="19" t="str">
         <x:v>[转述] 付费后简单任务仍浪费时间</x:v>
       </x:c>
-      <x:c r="AC11" s="19" t="str">
+      <x:c r="AE11" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD11" s="19" t="str">
+      <x:c r="AF11" s="19" t="str">
         <x:v>任务不可识别；非 Cowork 特性</x:v>
       </x:c>
-      <x:c r="AE11" s="19" t="str"/>
-      <x:c r="AF11" s="19" t="str">
+      <x:c r="AG11" s="19" t="str"/>
+      <x:c r="AH11" s="19" t="str">
         <x:v>用于说明国家明确也不等于内容合格</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="74" customHeight="1">
+    <x:row r="12" ht="82" customHeight="1">
       <x:c r="A12" s="19" t="str">
         <x:v>FB-ARE-20250912-000008</x:v>
       </x:c>
@@ -4402,18 +4458,24 @@
         <x:v>Manual indexed discovery + paraphrase</x:v>
       </x:c>
       <x:c r="AB12" s="19" t="str">
+        <x:v>I live in Dubai</x:v>
+      </x:c>
+      <x:c r="AC12" s="19" t="str">
+        <x:v>我住在迪拜。</x:v>
+      </x:c>
+      <x:c r="AD12" s="19" t="str">
         <x:v>[转述] Dubai 用户用 Comet 自动化邮件与本地购物研究</x:v>
       </x:c>
-      <x:c r="AC12" s="19" t="str">
+      <x:c r="AE12" s="19" t="str">
         <x:v>Included-Core</x:v>
       </x:c>
-      <x:c r="AD12" s="19" t="str"/>
-      <x:c r="AE12" s="19" t="str"/>
-      <x:c r="AF12" s="19" t="str">
+      <x:c r="AF12" s="19" t="str"/>
+      <x:c r="AG12" s="19" t="str"/>
+      <x:c r="AH12" s="19" t="str">
         <x:v>本轮最完整的地理+任务+替代链路样本</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="74" customHeight="1">
+    <x:row r="13" ht="82" customHeight="1">
       <x:c r="A13" s="19" t="str">
         <x:v>FB-ARE-20250322-000009</x:v>
       </x:c>
@@ -4493,21 +4555,23 @@
       <x:c r="AA13" s="19" t="str">
         <x:v>Manual indexed discovery + paraphrase</x:v>
       </x:c>
-      <x:c r="AB13" s="19" t="str">
+      <x:c r="AB13" s="19" t="str"/>
+      <x:c r="AC13" s="19" t="str"/>
+      <x:c r="AD13" s="19" t="str">
         <x:v>[转述] 询问 Dubai 可用的 Perplexity/Claude 优惠</x:v>
       </x:c>
-      <x:c r="AC13" s="19" t="str">
+      <x:c r="AE13" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD13" s="19" t="str">
+      <x:c r="AF13" s="19" t="str">
         <x:v>早于主窗口；更适合 05 国家需求</x:v>
       </x:c>
-      <x:c r="AE13" s="19" t="str"/>
-      <x:c r="AF13" s="19" t="str">
+      <x:c r="AG13" s="19" t="str"/>
+      <x:c r="AH13" s="19" t="str">
         <x:v>后续可转移到 demand signal 表</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="74" customHeight="1">
+    <x:row r="14" ht="82" customHeight="1">
       <x:c r="A14" s="19" t="str">
         <x:v>FB-ARE-20260404-000010</x:v>
       </x:c>
@@ -4586,18 +4650,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB14" s="19" t="str">
+        <x:v>one year subscription</x:v>
+      </x:c>
+      <x:c r="AC14" s="19" t="str">
+        <x:v>一年期订阅。</x:v>
+      </x:c>
+      <x:c r="AD14" s="19" t="str">
         <x:v>[转述] 年订阅后才发现图片、PPT、音乐仍受积分限制</x:v>
       </x:c>
-      <x:c r="AC14" s="19" t="str">
+      <x:c r="AE14" s="19" t="str">
         <x:v>Included-Core-LowGeo</x:v>
       </x:c>
-      <x:c r="AD14" s="19" t="str"/>
-      <x:c r="AE14" s="19" t="str"/>
-      <x:c r="AF14" s="19" t="str">
+      <x:c r="AF14" s="19" t="str"/>
+      <x:c r="AG14" s="19" t="str"/>
+      <x:c r="AH14" s="19" t="str">
         <x:v>只可用于 UAE 假设池，不能单独代表 UAE 用户</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="74" customHeight="1">
+    <x:row r="15" ht="82" customHeight="1">
       <x:c r="A15" s="19" t="str">
         <x:v>FB-ARE-20260220-000011</x:v>
       </x:c>
@@ -4676,18 +4746,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB15" s="19" t="str">
+        <x:v>very difficult to use</x:v>
+      </x:c>
+      <x:c r="AC15" s="19" t="str">
+        <x:v>非常难用。</x:v>
+      </x:c>
+      <x:c r="AD15" s="19" t="str">
         <x:v>[转述] 难上手、每次提问都耗 token，倾向改用 ChatGPT</x:v>
       </x:c>
-      <x:c r="AC15" s="19" t="str">
+      <x:c r="AE15" s="19" t="str">
         <x:v>Included-Core-MediumGeo</x:v>
       </x:c>
-      <x:c r="AD15" s="19" t="str"/>
-      <x:c r="AE15" s="19" t="str"/>
-      <x:c r="AF15" s="19" t="str">
+      <x:c r="AF15" s="19" t="str"/>
+      <x:c r="AG15" s="19" t="str"/>
+      <x:c r="AH15" s="19" t="str">
         <x:v>用户名不是可靠身份证据，仍不可升级为 High</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="74" customHeight="1">
+    <x:row r="16" ht="82" customHeight="1">
       <x:c r="A16" s="19" t="str">
         <x:v>FB-ARE-20260417-000012</x:v>
       </x:c>
@@ -4766,18 +4842,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB16" s="19" t="str">
+        <x:v>unable to use it</x:v>
+      </x:c>
+      <x:c r="AC16" s="19" t="str">
+        <x:v>无法继续使用。</x:v>
+      </x:c>
+      <x:c r="AD16" s="19" t="str">
         <x:v>[转述] 购买不到一个月即无法使用，并决定停用</x:v>
       </x:c>
-      <x:c r="AC16" s="19" t="str">
+      <x:c r="AE16" s="19" t="str">
         <x:v>Included-Core-LowGeo</x:v>
       </x:c>
-      <x:c r="AD16" s="19" t="str"/>
-      <x:c r="AE16" s="19" t="str"/>
-      <x:c r="AF16" s="19" t="str">
+      <x:c r="AF16" s="19" t="str"/>
+      <x:c r="AG16" s="19" t="str"/>
+      <x:c r="AH16" s="19" t="str">
         <x:v>任务细节一般，但付费—可用性—流失链路清楚</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="74" customHeight="1">
+    <x:row r="17" ht="82" customHeight="1">
       <x:c r="A17" s="19" t="str">
         <x:v>FB-ARE-20260416-000013</x:v>
       </x:c>
@@ -4854,18 +4936,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB17" s="19" t="str">
+        <x:v>Arabic language mistakes</x:v>
+      </x:c>
+      <x:c r="AC17" s="19" t="str">
+        <x:v>阿拉伯语错误。</x:v>
+      </x:c>
+      <x:c r="AD17" s="19" t="str">
         <x:v>[转述] 阿语错误较多，同时认为价格偏高</x:v>
       </x:c>
-      <x:c r="AC17" s="19" t="str">
+      <x:c r="AE17" s="19" t="str">
         <x:v>Included-Core-MediumGeo</x:v>
       </x:c>
-      <x:c r="AD17" s="19" t="str"/>
-      <x:c r="AE17" s="19" t="str"/>
-      <x:c r="AF17" s="19" t="str">
+      <x:c r="AF17" s="19" t="str"/>
+      <x:c r="AG17" s="19" t="str"/>
+      <x:c r="AH17" s="19" t="str">
         <x:v>本地化主题重要，但地理仍未独立验证</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="74" customHeight="1">
+    <x:row r="18" ht="82" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>FB-ARE-20250516-000014</x:v>
       </x:c>
@@ -4946,18 +5034,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB18" s="19" t="str">
+        <x:v>it kept throwing errors</x:v>
+      </x:c>
+      <x:c r="AC18" s="19" t="str">
+        <x:v>它一直报错。</x:v>
+      </x:c>
+      <x:c r="AD18" s="19" t="str">
         <x:v>[转述] 服务反复报错仍扣积分，客服也未响应</x:v>
       </x:c>
-      <x:c r="AC18" s="19" t="str">
+      <x:c r="AE18" s="19" t="str">
         <x:v>Included-Core-LowGeo</x:v>
       </x:c>
-      <x:c r="AD18" s="19" t="str"/>
-      <x:c r="AE18" s="19" t="str"/>
-      <x:c r="AF18" s="19" t="str">
+      <x:c r="AF18" s="19" t="str"/>
+      <x:c r="AG18" s="19" t="str"/>
+      <x:c r="AH18" s="19" t="str">
         <x:v>内容很强，但 UAE 归属仅 Low</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="74" customHeight="1">
+    <x:row r="19" ht="82" customHeight="1">
       <x:c r="A19" s="19" t="str">
         <x:v>FB-ARE-20260419-000015</x:v>
       </x:c>
@@ -5036,18 +5130,24 @@
         <x:v>Manual storefront review + paraphrase</x:v>
       </x:c>
       <x:c r="AB19" s="19" t="str">
+        <x:v>A very simple task burned 510 credits</x:v>
+      </x:c>
+      <x:c r="AC19" s="19" t="str">
+        <x:v>一个非常简单的任务消耗了 510 积分。</x:v>
+      </x:c>
+      <x:c r="AD19" s="19" t="str">
         <x:v>[转述] 一个简单任务消耗 510 credits，认为不值得订阅</x:v>
       </x:c>
-      <x:c r="AC19" s="19" t="str">
+      <x:c r="AE19" s="19" t="str">
         <x:v>Included-Core-LowGeo</x:v>
       </x:c>
-      <x:c r="AD19" s="19" t="str"/>
-      <x:c r="AE19" s="19" t="str"/>
-      <x:c r="AF19" s="19" t="str">
+      <x:c r="AF19" s="19" t="str"/>
+      <x:c r="AG19" s="19" t="str"/>
+      <x:c r="AH19" s="19" t="str">
         <x:v>价格主题清晰；任务具体内容未知</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="74" customHeight="1">
+    <x:row r="20" ht="82" customHeight="1">
       <x:c r="A20" s="19" t="str">
         <x:v>FB-ARE-20260000-000016</x:v>
       </x:c>
@@ -5122,20 +5222,26 @@
         <x:v>Manual storefront geo-audit</x:v>
       </x:c>
       <x:c r="AB20" s="19" t="str">
+        <x:v>Afghanistan</x:v>
+      </x:c>
+      <x:c r="AC20" s="19" t="str">
+        <x:v>阿富汗。</x:v>
+      </x:c>
+      <x:c r="AD20" s="19" t="str">
         <x:v>[转述] 正文明确出现 Afghanistan，与 UAE storefront 冲突</x:v>
       </x:c>
-      <x:c r="AC20" s="19" t="str">
+      <x:c r="AE20" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD20" s="19" t="str">
+      <x:c r="AF20" s="19" t="str">
         <x:v>Wrong country; geo counterexample</x:v>
       </x:c>
-      <x:c r="AE20" s="19" t="str"/>
-      <x:c r="AF20" s="19" t="str">
+      <x:c r="AG20" s="19" t="str"/>
+      <x:c r="AH20" s="19" t="str">
         <x:v>直接证明 storefront 不能等同 reviewer country</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="74" customHeight="1">
+    <x:row r="21" ht="82" customHeight="1">
       <x:c r="A21" s="19" t="str">
         <x:v>FB-GLB-20260000-000017</x:v>
       </x:c>
@@ -5208,20 +5314,26 @@
         <x:v>Search discovery only</x:v>
       </x:c>
       <x:c r="AB21" s="19" t="str">
+        <x:v>قضيت شهرين مع Claude Cowork</x:v>
+      </x:c>
+      <x:c r="AC21" s="19" t="str">
+        <x:v>我使用 Claude Cowork 两个月。</x:v>
+      </x:c>
+      <x:c r="AD21" s="19" t="str">
         <x:v>[转述] 阿语 Cowork 体验内容，但无法归属 UAE</x:v>
       </x:c>
-      <x:c r="AC21" s="19" t="str">
+      <x:c r="AE21" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD21" s="19" t="str">
+      <x:c r="AF21" s="19" t="str">
         <x:v>No UAE geo evidence</x:v>
       </x:c>
-      <x:c r="AE21" s="19" t="str"/>
-      <x:c r="AF21" s="19" t="str">
+      <x:c r="AG21" s="19" t="str"/>
+      <x:c r="AH21" s="19" t="str">
         <x:v>可进入 Global-Arabic 候选池</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="74" customHeight="1">
+    <x:row r="22" ht="82" customHeight="1">
       <x:c r="A22" s="19" t="str">
         <x:v>FB-GLB-20260000-000018</x:v>
       </x:c>
@@ -5295,21 +5407,23 @@
       <x:c r="AA22" s="19" t="str">
         <x:v>Manual public-page review + paraphrase</x:v>
       </x:c>
-      <x:c r="AB22" s="19" t="str">
+      <x:c r="AB22" s="19" t="str"/>
+      <x:c r="AC22" s="19" t="str"/>
+      <x:c r="AD22" s="19" t="str">
         <x:v>[转述] 阿语评论提到积分成本与图片生成问题</x:v>
       </x:c>
-      <x:c r="AC22" s="19" t="str">
+      <x:c r="AE22" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD22" s="19" t="str">
+      <x:c r="AF22" s="19" t="str">
         <x:v>No UAE geo evidence</x:v>
       </x:c>
-      <x:c r="AE22" s="19" t="str"/>
-      <x:c r="AF22" s="19" t="str">
+      <x:c r="AG22" s="19" t="str"/>
+      <x:c r="AH22" s="19" t="str">
         <x:v>进入 Global-Arabic 主题池，不进入 ARE</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="74" customHeight="1">
+    <x:row r="23" ht="82" customHeight="1">
       <x:c r="A23" s="19" t="str">
         <x:v>DS-ARE-20260520-000019</x:v>
       </x:c>
@@ -5386,20 +5500,26 @@
         <x:v>Manual indexed discovery + paraphrase</x:v>
       </x:c>
       <x:c r="AB23" s="19" t="str">
+        <x:v>Has anyone here tested GEO / AI search visibility?</x:v>
+      </x:c>
+      <x:c r="AC23" s="19" t="str">
+        <x:v>这里有人测试过 GEO / AI 搜索可见性吗？</x:v>
+      </x:c>
+      <x:c r="AD23" s="19" t="str">
         <x:v>[转述] UAE SME 寻求 AI 搜索可见性方案</x:v>
       </x:c>
-      <x:c r="AC23" s="19" t="str">
+      <x:c r="AE23" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD23" s="19" t="str">
+      <x:c r="AF23" s="19" t="str">
         <x:v>Belongs to 05 country-demand dataset</x:v>
       </x:c>
-      <x:c r="AE23" s="19" t="str"/>
-      <x:c r="AF23" s="19" t="str">
+      <x:c r="AG23" s="19" t="str"/>
+      <x:c r="AH23" s="19" t="str">
         <x:v>这是 04 与 05 分流的示例</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="74" customHeight="1">
+    <x:row r="24" ht="82" customHeight="1">
       <x:c r="A24" s="19" t="str">
         <x:v>FB-ARE-20260000-000020</x:v>
       </x:c>
@@ -5476,23 +5596,29 @@
         <x:v>Search discovery only</x:v>
       </x:c>
       <x:c r="AB24" s="19" t="str">
+        <x:v>Manus AI Agent Review UAE 2026</x:v>
+      </x:c>
+      <x:c r="AC24" s="19" t="str">
+        <x:v>2026 年 UAE Manus AI Agent 评测。</x:v>
+      </x:c>
+      <x:c r="AD24" s="19" t="str">
         <x:v>[转述] 面向 UAE 的评测文章，但不是用户原始反馈</x:v>
       </x:c>
-      <x:c r="AC24" s="19" t="str">
+      <x:c r="AE24" s="19" t="str">
         <x:v>Excluded</x:v>
       </x:c>
-      <x:c r="AD24" s="19" t="str">
+      <x:c r="AF24" s="19" t="str">
         <x:v>Editorial/SEO, not user-generated feedback</x:v>
       </x:c>
-      <x:c r="AE24" s="19" t="str"/>
-      <x:c r="AF24" s="19" t="str">
+      <x:c r="AG24" s="19" t="str"/>
+      <x:c r="AH24" s="19" t="str">
         <x:v>只用于发现当地词与候选假设</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AF1"/>
-    <x:mergeCell ref="A2:AF2"/>
+    <x:mergeCell ref="A1:AH1"/>
+    <x:mergeCell ref="A2:AH2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="R5:R24">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="High"/>
@@ -5500,7 +5626,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra354efb4e5a648d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc1ed435db0046b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7376,7 +7502,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdae5c672125e43b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fb712f79ab04a95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8166,7 +8292,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5d6a85a71b34eba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ace603caf074108"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8411,7 +8537,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5938d9b3f3e49b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95ff3b1fad6644c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>